<commit_message>
2026-08-13 1449 project file browser, many small UI tweaks, Test generator rewritten Risk, Issue sections to be more plausible .gitignore updated to ignore R, safe, generated & synthetic directories and data files: .sqlite, .csv, .xlsx
</commit_message>
<xml_diff>
--- a/effect-of-multiple-estimators-on-estimate-quality.xlsx
+++ b/effect-of-multiple-estimators-on-estimate-quality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghar115\professional\risk\cost-risk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B12F955-256A-499C-A562-113FA3796683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C321AF51-1AFE-49F1-A55A-110F9F8B5408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30945" yWindow="3000" windowWidth="14490" windowHeight="18990" xr2:uid="{D0F0ABF3-778C-47B5-9FFF-BBC5683E691E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D0F0ABF3-778C-47B5-9FFF-BBC5683E691E}"/>
   </bookViews>
   <sheets>
     <sheet name="Multiple Estimators" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="70">
   <si>
     <t>Number of Estimators (n)</t>
   </si>
@@ -216,9 +216,6 @@
     <t>Section 4: Group Scaling Matrix</t>
   </si>
   <si>
-    <t>Probability of Hitting Target (C9)</t>
-  </si>
-  <si>
     <t># Standard Errors</t>
   </si>
   <si>
@@ -238,6 +235,21 @@
   </si>
   <si>
     <t>PERT Estimate (O+(4*M)+P)/6</t>
+  </si>
+  <si>
+    <t>Programme Manager</t>
+  </si>
+  <si>
+    <t>Lead SME</t>
+  </si>
+  <si>
+    <t>Junior SME</t>
+  </si>
+  <si>
+    <t>Normal Distribution Facts</t>
+  </si>
+  <si>
+    <t>Probability of Hitting Target (C11)</t>
   </si>
 </sst>
 </file>
@@ -390,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -399,10 +411,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -471,16 +479,18 @@
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -821,397 +831,400 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" customWidth="1"/>
-    <col min="2" max="2" width="27" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27" style="13" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="12.28515625" style="3" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="26" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="29">
+      <c r="C2" s="27">
         <v>10</v>
       </c>
-      <c r="D2" s="29">
+      <c r="D2" s="27">
         <v>14</v>
       </c>
-      <c r="E2" s="29">
+      <c r="E2" s="27">
         <v>22</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="18">
         <f>(C2+(4*D2)+E2)/6</f>
         <v>14.666666666666666</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="29">
+      <c r="B3" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="27">
         <v>12</v>
       </c>
-      <c r="D3" s="29">
-        <v>15</v>
-      </c>
-      <c r="E3" s="29">
+      <c r="D3" s="27">
+        <v>15</v>
+      </c>
+      <c r="E3" s="27">
         <v>24</v>
       </c>
-      <c r="F3" s="20">
+      <c r="F3" s="18">
         <f t="shared" ref="F3:F5" si="0">(C3+(4*D3)+E3)/6</f>
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="29">
+      <c r="B4" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="27">
         <v>8</v>
       </c>
-      <c r="D4" s="29">
+      <c r="D4" s="27">
         <v>18</v>
       </c>
-      <c r="E4" s="29">
+      <c r="E4" s="27">
         <v>30</v>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="18">
         <f t="shared" si="0"/>
         <v>18.333333333333332</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="18">
         <f>AVERAGE(C2:C4)</f>
         <v>10</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="18">
         <f>AVERAGE(D2:D4)</f>
         <v>15.666666666666666</v>
       </c>
-      <c r="E5" s="20">
+      <c r="E5" s="18">
         <f>AVERAGE(E2:E4)</f>
         <v>25.333333333333332</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="18">
         <f t="shared" si="0"/>
         <v>16.333333333333332</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="19"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
     </row>
     <row r="7" spans="1:6" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="21" t="s">
+      <c r="A8" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="18">
         <f>(C5+(4*D5)+E5)/6</f>
         <v>16.333333333333332</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="21" t="s">
+      <c r="A9" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="18">
         <f>(E5-C5)/6</f>
         <v>2.5555555555555554</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
     </row>
     <row r="11" spans="1:6" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="27">
+        <f>C8*1.1</f>
+        <v>17.966666666666669</v>
+      </c>
+      <c r="D11" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+    </row>
+    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="28">
+        <v>0.95</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="30">
-        <v>18</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-    </row>
-    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="31">
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+    </row>
+    <row r="13" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="14"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+    </row>
+    <row r="14" spans="1:6" s="1" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="20"/>
+      <c r="B14" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+    </row>
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="22"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="23">
+        <v>0.68200000000000005</v>
+      </c>
+      <c r="D15" s="19">
+        <v>1</v>
+      </c>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+    </row>
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="22"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="23">
+        <v>0.9</v>
+      </c>
+      <c r="D16" s="19">
+        <v>1.64</v>
+      </c>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+    </row>
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="23">
         <v>0.95</v>
       </c>
-      <c r="D12" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-    </row>
-    <row r="13" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-    </row>
-    <row r="14" spans="1:6" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="22"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="24"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="25">
-        <v>0.68200000000000005</v>
-      </c>
-      <c r="D15" s="21">
-        <v>1</v>
-      </c>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="24"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="25">
-        <v>0.9</v>
-      </c>
-      <c r="D16" s="21">
-        <v>1.64</v>
-      </c>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="24"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="25">
-        <v>0.95</v>
-      </c>
-      <c r="D17" s="21">
+      <c r="D17" s="19">
         <v>1.96</v>
       </c>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="24"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="25">
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+    </row>
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="23">
         <v>0.997</v>
       </c>
-      <c r="D18" s="21">
+      <c r="D18" s="19">
         <v>3</v>
       </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26">
+      <c r="E18" s="24"/>
+      <c r="F18" s="24">
         <f>VLOOKUP($C$12,$C$15:$D$18,2,1)</f>
         <v>1.96</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
     </row>
     <row r="20" spans="1:6" s="1" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>58</v>
+      <c r="F20" s="16" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
-      <c r="B21" s="21">
+      <c r="A21" s="17"/>
+      <c r="B21" s="19">
         <v>1</v>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="18">
         <f>$C$9/SQRT(B21)</f>
         <v>2.5555555555555554</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="18">
         <f>$C$8-(VLOOKUP($C$12,$C$15:$D$18,2,1)*C21)</f>
         <v>11.324444444444444</v>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="18">
         <f>$C$8+(VLOOKUP($C$12,$C$15:$D$18,2,1)*C21)</f>
         <v>21.342222222222219</v>
       </c>
-      <c r="F21" s="27">
+      <c r="F21" s="25">
         <f>NORMDIST($C$11,$C$8,C21,TRUE)</f>
-        <v>0.74285550664195421</v>
+        <v>0.73863095883584196</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
-      <c r="B22" s="21">
+      <c r="A22" s="17"/>
+      <c r="B22" s="19">
         <v>3</v>
       </c>
-      <c r="C22" s="20">
+      <c r="C22" s="18">
         <f>$C$9/SQRT(B22)</f>
         <v>1.4754506879290437</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="18">
         <f>$C$8-(VLOOKUP($C$12,$C$15:$D$18,2,1)*C22)</f>
         <v>13.441449984992406</v>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="18">
         <f>$C$8+(VLOOKUP($C$12,$C$15:$D$18,2,1)*C22)</f>
         <v>19.225216681674258</v>
       </c>
-      <c r="F22" s="27">
+      <c r="F22" s="25">
         <f>NORMDIST($C$11,$C$8,C22,TRUE)</f>
-        <v>0.87067724728631402</v>
+        <v>0.86585441626565851</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
-      <c r="B23" s="21">
+      <c r="A23" s="17"/>
+      <c r="B23" s="19">
         <v>5</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="18">
         <f>$C$9/SQRT(B23)</f>
         <v>1.1428791884998923</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="18">
         <f>$C$8-(VLOOKUP($C$12,$C$15:$D$18,2,1)*C23)</f>
         <v>14.093290123873544</v>
       </c>
-      <c r="E23" s="20">
+      <c r="E23" s="18">
         <f>$C$8+(VLOOKUP($C$12,$C$15:$D$18,2,1)*C23)</f>
         <v>18.57337654279312</v>
       </c>
-      <c r="F23" s="27">
+      <c r="F23" s="25">
         <f>NORMDIST($C$11,$C$8,C23,TRUE)</f>
-        <v>0.9276217815947142</v>
+        <v>0.92351787114151296</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
-      <c r="B24" s="21">
+      <c r="A24" s="17"/>
+      <c r="B24" s="19">
         <v>10</v>
       </c>
-      <c r="C24" s="20">
+      <c r="C24" s="18">
         <f>$C$9/SQRT(B24)</f>
         <v>0.80813762426525237</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="18">
         <f>$C$8-(VLOOKUP($C$12,$C$15:$D$18,2,1)*C24)</f>
         <v>14.749383589773437</v>
       </c>
-      <c r="E24" s="20">
+      <c r="E24" s="18">
         <f>$C$8+(VLOOKUP($C$12,$C$15:$D$18,2,1)*C24)</f>
         <v>17.917283076893227</v>
       </c>
-      <c r="F24" s="27">
+      <c r="F24" s="25">
         <f>NORMDIST($C$11,$C$8,C24,TRUE)</f>
-        <v>0.98041302467465197</v>
+        <v>0.97836570141409251</v>
       </c>
     </row>
   </sheetData>
@@ -1230,7 +1243,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -1239,13 +1252,13 @@
       <c r="C1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="7" t="s">
         <v>43</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -1268,13 +1281,13 @@
       <c r="C2" s="2">
         <v>5</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="8">
         <v>10</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="2">
         <v>14</v>
       </c>
-      <c r="F2" s="11">
+      <c r="F2" s="9">
         <v>22</v>
       </c>
       <c r="G2" s="2">
@@ -1300,13 +1313,13 @@
       <c r="C3" s="2">
         <v>4</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>12</v>
       </c>
-      <c r="E3" s="5">
-        <v>15</v>
-      </c>
-      <c r="F3" s="11">
+      <c r="E3" s="2">
+        <v>15</v>
+      </c>
+      <c r="F3" s="9">
         <v>24</v>
       </c>
       <c r="G3" s="2">
@@ -1332,13 +1345,13 @@
       <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="2">
         <v>18</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="9">
         <v>30</v>
       </c>
       <c r="G4" s="2">
@@ -1365,15 +1378,15 @@
         <f>SUM(C2:C4)</f>
         <v>10</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="8">
         <f>AVERAGE(D2:D4)</f>
         <v>10</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="2">
         <f>AVERAGE(E2:E4)</f>
         <v>15.666666666666666</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="9">
         <f>AVERAGE(F2:F4)</f>
         <v>25.333333333333332</v>
       </c>
@@ -1394,30 +1407,30 @@
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="11"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="9"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="11" t="s">
+      <c r="D7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="9" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
@@ -1442,13 +1455,13 @@
         <f>(F5-D5)/6</f>
         <v>2.5555555555555554</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="11" t="s">
+      <c r="D8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>15</v>
       </c>
       <c r="G8" s="2" t="s">
@@ -1473,13 +1486,13 @@
         <f>(I5-G5)/6</f>
         <v>2.166666666666667</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="11" t="s">
+      <c r="D9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>15</v>
       </c>
       <c r="G9" s="2" t="s">
@@ -1496,27 +1509,27 @@
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="11"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="9"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="9" t="s">
         <v>37</v>
       </c>
       <c r="G11" s="2" t="s">
@@ -1536,15 +1549,15 @@
       <c r="C12" s="2">
         <v>1</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="8">
         <f>$C$8/SQRT(C12)</f>
         <v>2.5555555555555554</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="2">
         <f>$B$8-(1.96*D12)</f>
         <v>11.324444444444444</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="9">
         <f>$B$8+(1.96*D12)</f>
         <v>21.342222222222219</v>
       </c>
@@ -1568,15 +1581,15 @@
       <c r="C13" s="2">
         <v>3</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <f>$C$8/SQRT(C13)</f>
         <v>1.4754506879290437</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="2">
         <f>$B$8-(1.96*D13)</f>
         <v>13.441449984992406</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="9">
         <f>$B$8+(1.96*D13)</f>
         <v>19.225216681674258</v>
       </c>
@@ -1600,15 +1613,15 @@
       <c r="C14" s="2">
         <v>5</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="8">
         <f>$C$8/SQRT(C14)</f>
         <v>1.1428791884998923</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="2">
         <f>$B$8-(1.96*D14)</f>
         <v>14.093290123873544</v>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="9">
         <f>$B$8+(1.96*D14)</f>
         <v>18.57337654279312</v>
       </c>
@@ -1632,15 +1645,15 @@
       <c r="C15" s="2">
         <v>10</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="10">
         <f>$C$8/SQRT(C15)</f>
         <v>0.80813762426525237</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="11">
         <f>$B$8-(1.96*D15)</f>
         <v>14.749383589773437</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="12">
         <f>$B$8+(1.96*D15)</f>
         <v>17.917283076893227</v>
       </c>

</xml_diff>

<commit_message>
2026-08-13 1549 more UI tweaks.
2026-08-13 1449 project file browser, many small UI tweaks,
Test generator rewritten Risk, Issue sections to be more plausible
.gitignore updated to ignore R, safe, generated & synthetic directories
and data files: .sqlite, .csv, .xlsx
</commit_message>
<xml_diff>
--- a/effect-of-multiple-estimators-on-estimate-quality.xlsx
+++ b/effect-of-multiple-estimators-on-estimate-quality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghar115\professional\risk\cost-risk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B12F955-256A-499C-A562-113FA3796683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C321AF51-1AFE-49F1-A55A-110F9F8B5408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30945" yWindow="3000" windowWidth="14490" windowHeight="18990" xr2:uid="{D0F0ABF3-778C-47B5-9FFF-BBC5683E691E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D0F0ABF3-778C-47B5-9FFF-BBC5683E691E}"/>
   </bookViews>
   <sheets>
     <sheet name="Multiple Estimators" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="70">
   <si>
     <t>Number of Estimators (n)</t>
   </si>
@@ -216,9 +216,6 @@
     <t>Section 4: Group Scaling Matrix</t>
   </si>
   <si>
-    <t>Probability of Hitting Target (C9)</t>
-  </si>
-  <si>
     <t># Standard Errors</t>
   </si>
   <si>
@@ -238,6 +235,21 @@
   </si>
   <si>
     <t>PERT Estimate (O+(4*M)+P)/6</t>
+  </si>
+  <si>
+    <t>Programme Manager</t>
+  </si>
+  <si>
+    <t>Lead SME</t>
+  </si>
+  <si>
+    <t>Junior SME</t>
+  </si>
+  <si>
+    <t>Normal Distribution Facts</t>
+  </si>
+  <si>
+    <t>Probability of Hitting Target (C11)</t>
   </si>
 </sst>
 </file>
@@ -390,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -399,10 +411,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -471,16 +479,18 @@
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -821,397 +831,400 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" customWidth="1"/>
-    <col min="2" max="2" width="27" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27" style="13" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="12.28515625" style="3" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="26" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="29">
+      <c r="C2" s="27">
         <v>10</v>
       </c>
-      <c r="D2" s="29">
+      <c r="D2" s="27">
         <v>14</v>
       </c>
-      <c r="E2" s="29">
+      <c r="E2" s="27">
         <v>22</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="18">
         <f>(C2+(4*D2)+E2)/6</f>
         <v>14.666666666666666</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="29">
+      <c r="B3" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="27">
         <v>12</v>
       </c>
-      <c r="D3" s="29">
-        <v>15</v>
-      </c>
-      <c r="E3" s="29">
+      <c r="D3" s="27">
+        <v>15</v>
+      </c>
+      <c r="E3" s="27">
         <v>24</v>
       </c>
-      <c r="F3" s="20">
+      <c r="F3" s="18">
         <f t="shared" ref="F3:F5" si="0">(C3+(4*D3)+E3)/6</f>
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="29">
+      <c r="B4" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="27">
         <v>8</v>
       </c>
-      <c r="D4" s="29">
+      <c r="D4" s="27">
         <v>18</v>
       </c>
-      <c r="E4" s="29">
+      <c r="E4" s="27">
         <v>30</v>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="18">
         <f t="shared" si="0"/>
         <v>18.333333333333332</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="18">
         <f>AVERAGE(C2:C4)</f>
         <v>10</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="18">
         <f>AVERAGE(D2:D4)</f>
         <v>15.666666666666666</v>
       </c>
-      <c r="E5" s="20">
+      <c r="E5" s="18">
         <f>AVERAGE(E2:E4)</f>
         <v>25.333333333333332</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="18">
         <f t="shared" si="0"/>
         <v>16.333333333333332</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="19"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
     </row>
     <row r="7" spans="1:6" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="21" t="s">
+      <c r="A8" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="18">
         <f>(C5+(4*D5)+E5)/6</f>
         <v>16.333333333333332</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="21" t="s">
+      <c r="A9" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="18">
         <f>(E5-C5)/6</f>
         <v>2.5555555555555554</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
     </row>
     <row r="11" spans="1:6" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="27">
+        <f>C8*1.1</f>
+        <v>17.966666666666669</v>
+      </c>
+      <c r="D11" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+    </row>
+    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="28">
+        <v>0.95</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="30">
-        <v>18</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-    </row>
-    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="31">
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+    </row>
+    <row r="13" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="14"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+    </row>
+    <row r="14" spans="1:6" s="1" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="20"/>
+      <c r="B14" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+    </row>
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="22"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="23">
+        <v>0.68200000000000005</v>
+      </c>
+      <c r="D15" s="19">
+        <v>1</v>
+      </c>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+    </row>
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="22"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="23">
+        <v>0.9</v>
+      </c>
+      <c r="D16" s="19">
+        <v>1.64</v>
+      </c>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+    </row>
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="23">
         <v>0.95</v>
       </c>
-      <c r="D12" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-    </row>
-    <row r="13" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-    </row>
-    <row r="14" spans="1:6" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="22"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="24"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="25">
-        <v>0.68200000000000005</v>
-      </c>
-      <c r="D15" s="21">
-        <v>1</v>
-      </c>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="24"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="25">
-        <v>0.9</v>
-      </c>
-      <c r="D16" s="21">
-        <v>1.64</v>
-      </c>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="24"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="25">
-        <v>0.95</v>
-      </c>
-      <c r="D17" s="21">
+      <c r="D17" s="19">
         <v>1.96</v>
       </c>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="24"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="25">
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+    </row>
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="23">
         <v>0.997</v>
       </c>
-      <c r="D18" s="21">
+      <c r="D18" s="19">
         <v>3</v>
       </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26">
+      <c r="E18" s="24"/>
+      <c r="F18" s="24">
         <f>VLOOKUP($C$12,$C$15:$D$18,2,1)</f>
         <v>1.96</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
     </row>
     <row r="20" spans="1:6" s="1" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>58</v>
+      <c r="F20" s="16" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
-      <c r="B21" s="21">
+      <c r="A21" s="17"/>
+      <c r="B21" s="19">
         <v>1</v>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="18">
         <f>$C$9/SQRT(B21)</f>
         <v>2.5555555555555554</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="18">
         <f>$C$8-(VLOOKUP($C$12,$C$15:$D$18,2,1)*C21)</f>
         <v>11.324444444444444</v>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="18">
         <f>$C$8+(VLOOKUP($C$12,$C$15:$D$18,2,1)*C21)</f>
         <v>21.342222222222219</v>
       </c>
-      <c r="F21" s="27">
+      <c r="F21" s="25">
         <f>NORMDIST($C$11,$C$8,C21,TRUE)</f>
-        <v>0.74285550664195421</v>
+        <v>0.73863095883584196</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
-      <c r="B22" s="21">
+      <c r="A22" s="17"/>
+      <c r="B22" s="19">
         <v>3</v>
       </c>
-      <c r="C22" s="20">
+      <c r="C22" s="18">
         <f>$C$9/SQRT(B22)</f>
         <v>1.4754506879290437</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="18">
         <f>$C$8-(VLOOKUP($C$12,$C$15:$D$18,2,1)*C22)</f>
         <v>13.441449984992406</v>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="18">
         <f>$C$8+(VLOOKUP($C$12,$C$15:$D$18,2,1)*C22)</f>
         <v>19.225216681674258</v>
       </c>
-      <c r="F22" s="27">
+      <c r="F22" s="25">
         <f>NORMDIST($C$11,$C$8,C22,TRUE)</f>
-        <v>0.87067724728631402</v>
+        <v>0.86585441626565851</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
-      <c r="B23" s="21">
+      <c r="A23" s="17"/>
+      <c r="B23" s="19">
         <v>5</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="18">
         <f>$C$9/SQRT(B23)</f>
         <v>1.1428791884998923</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="18">
         <f>$C$8-(VLOOKUP($C$12,$C$15:$D$18,2,1)*C23)</f>
         <v>14.093290123873544</v>
       </c>
-      <c r="E23" s="20">
+      <c r="E23" s="18">
         <f>$C$8+(VLOOKUP($C$12,$C$15:$D$18,2,1)*C23)</f>
         <v>18.57337654279312</v>
       </c>
-      <c r="F23" s="27">
+      <c r="F23" s="25">
         <f>NORMDIST($C$11,$C$8,C23,TRUE)</f>
-        <v>0.9276217815947142</v>
+        <v>0.92351787114151296</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
-      <c r="B24" s="21">
+      <c r="A24" s="17"/>
+      <c r="B24" s="19">
         <v>10</v>
       </c>
-      <c r="C24" s="20">
+      <c r="C24" s="18">
         <f>$C$9/SQRT(B24)</f>
         <v>0.80813762426525237</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="18">
         <f>$C$8-(VLOOKUP($C$12,$C$15:$D$18,2,1)*C24)</f>
         <v>14.749383589773437</v>
       </c>
-      <c r="E24" s="20">
+      <c r="E24" s="18">
         <f>$C$8+(VLOOKUP($C$12,$C$15:$D$18,2,1)*C24)</f>
         <v>17.917283076893227</v>
       </c>
-      <c r="F24" s="27">
+      <c r="F24" s="25">
         <f>NORMDIST($C$11,$C$8,C24,TRUE)</f>
-        <v>0.98041302467465197</v>
+        <v>0.97836570141409251</v>
       </c>
     </row>
   </sheetData>
@@ -1230,7 +1243,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -1239,13 +1252,13 @@
       <c r="C1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="7" t="s">
         <v>43</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -1268,13 +1281,13 @@
       <c r="C2" s="2">
         <v>5</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="8">
         <v>10</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="2">
         <v>14</v>
       </c>
-      <c r="F2" s="11">
+      <c r="F2" s="9">
         <v>22</v>
       </c>
       <c r="G2" s="2">
@@ -1300,13 +1313,13 @@
       <c r="C3" s="2">
         <v>4</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>12</v>
       </c>
-      <c r="E3" s="5">
-        <v>15</v>
-      </c>
-      <c r="F3" s="11">
+      <c r="E3" s="2">
+        <v>15</v>
+      </c>
+      <c r="F3" s="9">
         <v>24</v>
       </c>
       <c r="G3" s="2">
@@ -1332,13 +1345,13 @@
       <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="2">
         <v>18</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="9">
         <v>30</v>
       </c>
       <c r="G4" s="2">
@@ -1365,15 +1378,15 @@
         <f>SUM(C2:C4)</f>
         <v>10</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="8">
         <f>AVERAGE(D2:D4)</f>
         <v>10</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="2">
         <f>AVERAGE(E2:E4)</f>
         <v>15.666666666666666</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="9">
         <f>AVERAGE(F2:F4)</f>
         <v>25.333333333333332</v>
       </c>
@@ -1394,30 +1407,30 @@
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="11"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="9"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="11" t="s">
+      <c r="D7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="9" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
@@ -1442,13 +1455,13 @@
         <f>(F5-D5)/6</f>
         <v>2.5555555555555554</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="11" t="s">
+      <c r="D8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>15</v>
       </c>
       <c r="G8" s="2" t="s">
@@ -1473,13 +1486,13 @@
         <f>(I5-G5)/6</f>
         <v>2.166666666666667</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="11" t="s">
+      <c r="D9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>15</v>
       </c>
       <c r="G9" s="2" t="s">
@@ -1496,27 +1509,27 @@
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="11"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="9"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="9" t="s">
         <v>37</v>
       </c>
       <c r="G11" s="2" t="s">
@@ -1536,15 +1549,15 @@
       <c r="C12" s="2">
         <v>1</v>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="8">
         <f>$C$8/SQRT(C12)</f>
         <v>2.5555555555555554</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="2">
         <f>$B$8-(1.96*D12)</f>
         <v>11.324444444444444</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="9">
         <f>$B$8+(1.96*D12)</f>
         <v>21.342222222222219</v>
       </c>
@@ -1568,15 +1581,15 @@
       <c r="C13" s="2">
         <v>3</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="8">
         <f>$C$8/SQRT(C13)</f>
         <v>1.4754506879290437</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="2">
         <f>$B$8-(1.96*D13)</f>
         <v>13.441449984992406</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="9">
         <f>$B$8+(1.96*D13)</f>
         <v>19.225216681674258</v>
       </c>
@@ -1600,15 +1613,15 @@
       <c r="C14" s="2">
         <v>5</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="8">
         <f>$C$8/SQRT(C14)</f>
         <v>1.1428791884998923</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="2">
         <f>$B$8-(1.96*D14)</f>
         <v>14.093290123873544</v>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="9">
         <f>$B$8+(1.96*D14)</f>
         <v>18.57337654279312</v>
       </c>
@@ -1632,15 +1645,15 @@
       <c r="C15" s="2">
         <v>10</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="10">
         <f>$C$8/SQRT(C15)</f>
         <v>0.80813762426525237</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="11">
         <f>$B$8-(1.96*D15)</f>
         <v>14.749383589773437</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="12">
         <f>$B$8+(1.96*D15)</f>
         <v>17.917283076893227</v>
       </c>

</xml_diff>